<commit_message>
revising launch sh files
</commit_message>
<xml_diff>
--- a/applications/SHIELD/Documentation/PS Syphilis - Cases by Sex and Sex of Sex Partners (US 2015-2024).xlsx
+++ b/applications/SHIELD/Documentation/PS Syphilis - Cases by Sex and Sex of Sex Partners (US 2015-2024).xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://livejohnshopkins-my.sharepoint.com/personal/pkasaie1_jh_edu/Documents/SHIELDR01/Simulation/code/jheem_analyses/applications/SHIELD/Documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="54" documentId="13_ncr:1_{A0F7102C-F699-B042-A64E-207DB11C90FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{23D90AD4-FCD4-3B45-9171-A86A250AF0D4}"/>
+  <xr:revisionPtr revIDLastSave="56" documentId="13_ncr:1_{A0F7102C-F699-B042-A64E-207DB11C90FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88B646EE-30FE-2949-818F-5DC08637FFE1}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="34560" windowHeight="19520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="76580" yWindow="600" windowWidth="38400" windowHeight="19520" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="3" r:id="rId2"/>
-    <sheet name="CA" sheetId="4" r:id="rId3"/>
+    <sheet name="Sheet2" sheetId="6" r:id="rId3"/>
+    <sheet name="CA" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Sheet1!$A$5:$H$59</definedName>
@@ -3750,6 +3751,22 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE604CA6-5D88-0144-B08A-91DBBAA3536C}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1">
+        <f>2395*12</f>
+        <v>28740</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{256FC72E-A572-7D4B-A75E-263A2A9F0674}">
   <dimension ref="B1:M48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>

</xml_diff>

<commit_message>
fixing the calibration plot code inconsistencies
</commit_message>
<xml_diff>
--- a/applications/SHIELD/Documentation/PS Syphilis - Cases by Sex and Sex of Sex Partners (US 2015-2024).xlsx
+++ b/applications/SHIELD/Documentation/PS Syphilis - Cases by Sex and Sex of Sex Partners (US 2015-2024).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://livejohnshopkins-my.sharepoint.com/personal/pkasaie1_jh_edu/Documents/SHIELDR01/Simulation/code/jheem_analyses/applications/SHIELD/Documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="56" documentId="13_ncr:1_{A0F7102C-F699-B042-A64E-207DB11C90FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88B646EE-30FE-2949-818F-5DC08637FFE1}"/>
+  <xr:revisionPtr revIDLastSave="57" documentId="13_ncr:1_{A0F7102C-F699-B042-A64E-207DB11C90FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ADEF3F69-C8C5-7A4B-B8DF-59FF261C779A}"/>
   <bookViews>
     <workbookView xWindow="76580" yWindow="600" windowWidth="38400" windowHeight="19520" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3752,13 +3752,19 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE604CA6-5D88-0144-B08A-91DBBAA3536C}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1">
         <f>2395*12</f>
         <v>28740</v>
+      </c>
+    </row>
+    <row r="32" spans="6:6">
+      <c r="F32">
+        <f>2096695381/737690966</f>
+        <v>2.8422408266282062</v>
       </c>
     </row>
   </sheetData>

</xml_diff>